<commit_message>
Updated Zergaw_territory_revenue_chart with updated work
</commit_message>
<xml_diff>
--- a/Zergaw_territory_revenue_chart.xlsx
+++ b/Zergaw_territory_revenue_chart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tihitinazergaw\Documents\DATA_Labs\Capstone_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{077CAFDE-B6AA-46E4-BBD2-CB39E8780A96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79FB57A2-E0CA-4A42-9916-E5B716087102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A1C97ABC-3D67-40A3-9C88-D5AE7397E28D}"/>
   </bookViews>
@@ -17,7 +17,7 @@
   </sheets>
   <calcPr calcId="0"/>
   <pivotCaches>
-    <pivotCache cacheId="7" r:id="rId2"/>
+    <pivotCache cacheId="0" r:id="rId2"/>
   </pivotCaches>
 </workbook>
 </file>
@@ -527,11 +527,14 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -2239,6 +2242,121 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>184150</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>88900</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>12700</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>82550</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="TextBox 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7BEB8543-5508-EC84-77C1-4B5BA105EBEC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2622550" y="8191500"/>
+          <a:ext cx="5791200" cy="914400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>This chart shows a seasonal pattern. August 2025 recorded</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>the highest revenue from 2022-202, followed by</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t> October 2025</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>.</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t> This increase was</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t> driven by both higher number of transactions and larger average transaction size.  Overall,</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>2025 shows</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t> the stronges performance while </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>May</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t> represents one of the lowest revenue periods. </a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2530,7 +2648,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9F2053FF-E9D4-4A30-85B2-CFB17BB05DAF}" name="PivotTable1" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9F2053FF-E9D4-4A30-85B2-CFB17BB05DAF}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
   <location ref="F11:K25" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField axis="axisCol" showAll="0">
@@ -3016,7 +3134,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FAA47F1-F862-471F-8BD6-1D17D52F3523}">
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:K52"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="6" max="6" width="12.453125" bestFit="1" customWidth="1"/>
@@ -3822,6 +3940,9 @@
         <v>22506.959999999999</v>
       </c>
     </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A52" s="3"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId2"/>

</xml_diff>

<commit_message>
Update Zergaw_territory_revenue_chart with updated work
</commit_message>
<xml_diff>
--- a/Zergaw_territory_revenue_chart.xlsx
+++ b/Zergaw_territory_revenue_chart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tihitinazergaw\Documents\DATA_Labs\Capstone_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79FB57A2-E0CA-4A42-9916-E5B716087102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF91A617-A773-43C8-B826-2676A5C116EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A1C97ABC-3D67-40A3-9C88-D5AE7397E28D}"/>
   </bookViews>
@@ -2313,7 +2313,7 @@
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100"/>
-            <a:t>the highest revenue from 2022-202, followed by</a:t>
+            <a:t>the highest revenue from 2022-2025, followed by</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" baseline="0"/>

</xml_diff>